<commit_message>
part user config 配置
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/zkb/partOrderUserConfig/Part_Order_User_Config_Template.xlsx
+++ b/src/src/main/webapp/portal/zkb/partOrderUserConfig/Part_Order_User_Config_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\503202755\Desktop\New folder (14)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D21123B-A545-4100-AC6A-7232E4EE863B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DC6895-E7A4-47A9-A431-5FC5B48CC7EA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -449,15 +449,15 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{108350D3-0B7D-4C08-AF27-C525A99AC6CA}">
       <formula1>"CS,CT,XR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{6728F639-C0B2-47EA-AE1B-83EAA32A6D0C}">
-      <formula1>"400公用邮箱,待技术支持审批,待经理审批,待开单,待下单,待归还,待关单,完成"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576" xr:uid="{DF829C73-846E-421D-B7A2-74E582595533}">
       <formula1>"是,否"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{FE8D1FEF-3E0A-40CE-9541-AA847DA37673}">
       <formula1>"Probe"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{EEE9FBDB-3935-4C71-A311-D94CD74EDAAD}">
+      <formula1>"400公共邮箱,技术支持,区域经理,400开单人,400下单人,GE Admin"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
USER CONFIG 导出 导入
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/zkb/partOrderUserConfig/Part_Order_User_Config_Template.xlsx
+++ b/src/src/main/webapp/portal/zkb/partOrderUserConfig/Part_Order_User_Config_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\503202755\Desktop\New folder (14)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\503202755\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109E51C3-3E05-4B74-8E14-79D0B6E428D0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31ED620-CA65-4F54-800F-454FE91ACABA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>名称</t>
   </si>
@@ -58,6 +58,15 @@
   </si>
   <si>
     <t>APM用户名</t>
+  </si>
+  <si>
+    <t>UsBackUp</t>
+  </si>
+  <si>
+    <t>是否删除</t>
+  </si>
+  <si>
+    <t>SYSTEM ID</t>
   </si>
 </sst>
 </file>
@@ -390,73 +399,84 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="21.21875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="25.44140625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="19.77734375" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" customWidth="1"/>
-    <col min="8" max="8" width="19.77734375" customWidth="1"/>
-    <col min="9" max="9" width="32" style="2" customWidth="1"/>
-    <col min="10" max="10" width="30.109375" customWidth="1"/>
-    <col min="11" max="11" width="41.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.44140625" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="25.44140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="21.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="19.77734375" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" customWidth="1"/>
+    <col min="9" max="10" width="19.77734375" customWidth="1"/>
+    <col min="11" max="11" width="32" style="2" customWidth="1"/>
+    <col min="12" max="12" width="30.109375" customWidth="1"/>
+    <col min="13" max="13" width="41.77734375" customWidth="1"/>
+    <col min="14" max="14" width="34.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{50DA0FCA-0A1A-4707-ADC4-E7DEF9686B03}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{50DA0FCA-0A1A-4707-ADC4-E7DEF9686B03}">
       <formula1>"North,South,East,West"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{108350D3-0B7D-4C08-AF27-C525A99AC6CA}">
-      <formula1>"CS,CT,XR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1048576" xr:uid="{DF829C73-846E-421D-B7A2-74E582595533}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:N1048576" xr:uid="{DF829C73-846E-421D-B7A2-74E582595533}">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{FE8D1FEF-3E0A-40CE-9541-AA847DA37673}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L1048576" xr:uid="{FE8D1FEF-3E0A-40CE-9541-AA847DA37673}">
       <formula1>"Probe"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{EEE9FBDB-3935-4C71-A311-D94CD74EDAAD}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{EEE9FBDB-3935-4C71-A311-D94CD74EDAAD}">
       <formula1>"400公共邮箱,技术支持,区域经理,400开单人,400下单人,GE Admin"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576" xr:uid="{B17C28DD-A5DF-472D-8EAA-1C421CD65100}">
+      <formula1>"US,CT,XR"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>